<commit_message>
Improved data analysis and comparison with FEM
</commit_message>
<xml_diff>
--- a/PH0__Allowables_and_Failure_Scenarios/Static_TEST__Data-Processing_UPDATED/phial_failure_summary.xlsx
+++ b/PH0__Allowables_and_Failure_Scenarios/Static_TEST__Data-Processing_UPDATED/phial_failure_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K77"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,35 +439,25 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Tangent_Modulus_N_per_mm</t>
+          <t>Failure_Load_N</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Fit_Intercept_N</t>
+          <t>Failure_Displacement_mm</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Fit_R2</t>
+          <t>Num_Peaks_Detected</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Window_Start_mm</t>
+          <t>All_Peak_Loads_N</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>Window_End_mm</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>N_Points_Used</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
@@ -491,24 +481,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>564.9089746884376</v>
+        <v>389.35</v>
       </c>
       <c r="F2" t="n">
-        <v>-208.4962472491393</v>
+        <v>1.0449</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9990066246859156</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.5273</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1.0428</v>
-      </c>
-      <c r="J2" t="n">
-        <v>387</v>
-      </c>
-      <c r="K2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>389.35</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -528,24 +514,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>722.2876454574543</v>
+        <v>458.03</v>
       </c>
       <c r="F3" t="n">
-        <v>-305.2449856564818</v>
+        <v>1.0707</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9990008038840762</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.4874</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1.004</v>
-      </c>
-      <c r="J3" t="n">
-        <v>387</v>
-      </c>
-      <c r="K3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>458.03</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -565,24 +547,20 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>505.8058678745455</v>
+        <v>207.95</v>
       </c>
       <c r="F4" t="n">
-        <v>-148.8721359743145</v>
+        <v>0.7067</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9990135976027035</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0.3764</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0.7056</v>
-      </c>
-      <c r="J4" t="n">
-        <v>246</v>
-      </c>
-      <c r="K4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>207.95</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -602,24 +580,20 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>395.9804155424945</v>
+        <v>138.2</v>
       </c>
       <c r="F5" t="n">
-        <v>-219.1109694854424</v>
+        <v>0.8907</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9990272898214905</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0.7563</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.8253</v>
-      </c>
-      <c r="J5" t="n">
-        <v>54</v>
-      </c>
-      <c r="K5" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>138.20</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -639,24 +613,20 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>634.6099417361892</v>
+        <v>271.88</v>
       </c>
       <c r="F6" t="n">
-        <v>-565.4297894708048</v>
+        <v>1.3014</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9990094798310554</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.9889</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1.2555</v>
-      </c>
-      <c r="J6" t="n">
-        <v>102</v>
-      </c>
-      <c r="K6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>271.88</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -676,24 +646,20 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>882.8195485462074</v>
+        <v>320.75</v>
       </c>
       <c r="F7" t="n">
-        <v>30.79492207277005</v>
+        <v>0.3437</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9990053455654037</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.2652</v>
-      </c>
-      <c r="J7" t="n">
-        <v>415</v>
-      </c>
-      <c r="K7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>320.75</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -713,24 +679,20 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>933.114568510945</v>
+        <v>339.61</v>
       </c>
       <c r="F8" t="n">
-        <v>-258.0776606905899</v>
+        <v>0.6613</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9990090152336888</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.3667</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.5518</v>
-      </c>
-      <c r="J8" t="n">
-        <v>140</v>
-      </c>
-      <c r="K8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>339.61</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -750,24 +712,20 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>888.5158403728543</v>
+        <v>213.57</v>
       </c>
       <c r="F9" t="n">
-        <v>-247.8456851731003</v>
+        <v>0.5182</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9990034203328388</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.3455</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.5178</v>
-      </c>
-      <c r="J9" t="n">
-        <v>256</v>
-      </c>
-      <c r="K9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>213.57</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -787,24 +745,20 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>690.4872108759761</v>
+        <v>245.91</v>
       </c>
       <c r="F10" t="n">
-        <v>-652.5924274850014</v>
+        <v>1.273</v>
       </c>
       <c r="G10" t="n">
-        <v>0.999085618749101</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1.0911</v>
-      </c>
-      <c r="I10" t="n">
-        <v>1.2123</v>
-      </c>
-      <c r="J10" t="n">
-        <v>49</v>
-      </c>
-      <c r="K10" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>245.91</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -824,28 +778,20 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>67.19889609175699</v>
+        <v>61.05</v>
       </c>
       <c r="F11" t="n">
-        <v>-17.89571021712781</v>
+        <v>1.2832</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9942112996175445</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.5197000000000001</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.5683</v>
-      </c>
-      <c r="J11" t="n">
-        <v>20</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>NO_WINDOW_MET_R2_THRESHOLD - relaxed to best available, verify manually</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>61.05, 209.82</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -865,24 +811,20 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1079.829710536142</v>
+        <v>261.24</v>
       </c>
       <c r="F12" t="n">
-        <v>-286.7735269055113</v>
+        <v>0.5053</v>
       </c>
       <c r="G12" t="n">
-        <v>0.9990529775959623</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.3155</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.5041</v>
-      </c>
-      <c r="J12" t="n">
-        <v>287</v>
-      </c>
-      <c r="K12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>261.24</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -902,24 +844,20 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>992.6551795107334</v>
+        <v>305.97</v>
       </c>
       <c r="F13" t="n">
-        <v>-550.3268915847461</v>
+        <v>0.8588</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9990376588065674</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.6242</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.8578</v>
-      </c>
-      <c r="J13" t="n">
-        <v>175</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>305.97</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -939,24 +877,20 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1254.173312050103</v>
+        <v>598.17</v>
       </c>
       <c r="F14" t="n">
-        <v>-135.4335513494566</v>
+        <v>0.5767</v>
       </c>
       <c r="G14" t="n">
-        <v>0.9990059717892407</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0.5760999999999999</v>
-      </c>
-      <c r="J14" t="n">
-        <v>700</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>598.17</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -976,24 +910,20 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>744.4551805627751</v>
+        <v>495.37</v>
       </c>
       <c r="F15" t="n">
-        <v>14.26215322770704</v>
+        <v>0.8105</v>
       </c>
       <c r="G15" t="n">
-        <v>0.9990583983407613</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.0308</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0.0825</v>
-      </c>
-      <c r="J15" t="n">
-        <v>39</v>
-      </c>
-      <c r="K15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>495.37</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1013,24 +943,20 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>940.3542275950794</v>
+        <v>307.97</v>
       </c>
       <c r="F16" t="n">
-        <v>-465.3802235908225</v>
+        <v>0.8082</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9990015546594063</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.5516</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0.7586000000000001</v>
-      </c>
-      <c r="J16" t="n">
-        <v>155</v>
-      </c>
-      <c r="K16" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>307.97, 227.00, 213.59</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1050,24 +976,20 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>521.2607588949054</v>
+        <v>220.19</v>
       </c>
       <c r="F17" t="n">
-        <v>-236.4540265697304</v>
+        <v>1.0053</v>
       </c>
       <c r="G17" t="n">
-        <v>0.9990072313109516</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.5901</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.7077</v>
-      </c>
-      <c r="J17" t="n">
-        <v>86</v>
-      </c>
-      <c r="K17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>220.19</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1087,24 +1009,20 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1108.720455713018</v>
+        <v>237.03</v>
       </c>
       <c r="F18" t="n">
-        <v>9.466241916215807</v>
+        <v>0.2063</v>
       </c>
       <c r="G18" t="n">
-        <v>0.999017640506608</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.0673</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0.2059</v>
-      </c>
-      <c r="J18" t="n">
-        <v>412</v>
-      </c>
-      <c r="K18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>237.03</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1124,24 +1042,20 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>992.5304053578541</v>
+        <v>290.68</v>
       </c>
       <c r="F19" t="n">
-        <v>-721.7389381388832</v>
+        <v>1.0173</v>
       </c>
       <c r="G19" t="n">
-        <v>0.9990296704043412</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0.8333</v>
-      </c>
-      <c r="I19" t="n">
-        <v>1.016</v>
-      </c>
-      <c r="J19" t="n">
-        <v>140</v>
-      </c>
-      <c r="K19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>290.68</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1161,24 +1075,20 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>270.5121708495141</v>
+        <v>127.12</v>
       </c>
       <c r="F20" t="n">
-        <v>-83.51872111659806</v>
+        <v>0.6588000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>0.9990048663698017</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0.3047</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0.5208</v>
-      </c>
-      <c r="J20" t="n">
-        <v>169</v>
-      </c>
-      <c r="K20" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>127.12, 65.75, 126.87</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1198,24 +1108,20 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>675.1827652792974</v>
+        <v>128.38</v>
       </c>
       <c r="F21" t="n">
-        <v>27.12774789226088</v>
+        <v>0.149</v>
       </c>
       <c r="G21" t="n">
-        <v>0.999003284436334</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0.0236</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.1483</v>
-      </c>
-      <c r="J21" t="n">
-        <v>190</v>
-      </c>
-      <c r="K21" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>128.38, 343.74</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1235,24 +1141,20 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>244.5182975752823</v>
+        <v>238.96</v>
       </c>
       <c r="F22" t="n">
-        <v>-126.5825146266304</v>
+        <v>0.8993</v>
       </c>
       <c r="G22" t="n">
-        <v>0.9991837300121431</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0.5073</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0.6574</v>
-      </c>
-      <c r="J22" t="n">
-        <v>56</v>
-      </c>
-      <c r="K22" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>238.96, 137.99, 138.90, 144.37, 459.31</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1272,24 +1174,20 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>652.1816695356932</v>
+        <v>368.47</v>
       </c>
       <c r="F23" t="n">
-        <v>-552.452458456257</v>
+        <v>1.3157</v>
       </c>
       <c r="G23" t="n">
-        <v>0.9990441358876112</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0.9358</v>
-      </c>
-      <c r="I23" t="n">
-        <v>1.1698</v>
-      </c>
-      <c r="J23" t="n">
-        <v>90</v>
-      </c>
-      <c r="K23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>368.47</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1309,24 +1207,20 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>942.5776133681314</v>
+        <v>202.01</v>
       </c>
       <c r="F24" t="n">
-        <v>-1319.157090744626</v>
+        <v>1.6131</v>
       </c>
       <c r="G24" t="n">
-        <v>0.9991649015031329</v>
-      </c>
-      <c r="H24" t="n">
-        <v>1.4715</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1.6099</v>
-      </c>
-      <c r="J24" t="n">
-        <v>54</v>
-      </c>
-      <c r="K24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>202.01</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1346,24 +1240,20 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1081.465636933423</v>
+        <v>302.9</v>
       </c>
       <c r="F25" t="n">
-        <v>-36.44938939694934</v>
+        <v>0.3117</v>
       </c>
       <c r="G25" t="n">
-        <v>0.999016002749457</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0.1123</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0.3111</v>
-      </c>
-      <c r="J25" t="n">
-        <v>298</v>
-      </c>
-      <c r="K25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>302.90</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1383,24 +1273,20 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>977.0848741258305</v>
+        <v>276.9</v>
       </c>
       <c r="F26" t="n">
-        <v>-683.4909711967898</v>
+        <v>0.9799</v>
       </c>
       <c r="G26" t="n">
-        <v>0.9990268853884482</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0.7634</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0.9785</v>
-      </c>
-      <c r="J26" t="n">
-        <v>157</v>
-      </c>
-      <c r="K26" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>276.90</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1420,24 +1306,20 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>1246.675590543702</v>
+        <v>355.59</v>
       </c>
       <c r="F27" t="n">
-        <v>-86.24073895902097</v>
+        <v>0.3444</v>
       </c>
       <c r="G27" t="n">
-        <v>0.9990000701681392</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0.1456</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="J27" t="n">
-        <v>347</v>
-      </c>
-      <c r="K27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>355.59</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1457,24 +1339,20 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>904.9977807171285</v>
+        <v>515.55</v>
       </c>
       <c r="F28" t="n">
-        <v>-259.3896980921248</v>
+        <v>0.8202</v>
       </c>
       <c r="G28" t="n">
-        <v>0.9990115459751795</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0.3526</v>
-      </c>
-      <c r="I28" t="n">
-        <v>0.506</v>
-      </c>
-      <c r="J28" t="n">
-        <v>156</v>
-      </c>
-      <c r="K28" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>515.55, 132.92, 385.58, 434.26, 442.68</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1494,24 +1372,20 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>317.5376228768287</v>
+        <v>134.79</v>
       </c>
       <c r="F29" t="n">
-        <v>-165.4738411717777</v>
+        <v>0.8919</v>
       </c>
       <c r="G29" t="n">
-        <v>0.9990857903252427</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0.6223</v>
-      </c>
-      <c r="I29" t="n">
-        <v>0.7725</v>
-      </c>
-      <c r="J29" t="n">
-        <v>78</v>
-      </c>
-      <c r="K29" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>134.79</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1531,24 +1405,20 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1190.861216640523</v>
+        <v>293.17</v>
       </c>
       <c r="F30" t="n">
-        <v>-735.7721143103753</v>
+        <v>0.8578</v>
       </c>
       <c r="G30" t="n">
-        <v>0.9990075829902783</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0.7147</v>
-      </c>
-      <c r="I30" t="n">
-        <v>0.847</v>
-      </c>
-      <c r="J30" t="n">
-        <v>139</v>
-      </c>
-      <c r="K30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>293.17</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1568,24 +1438,20 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1049.309642057045</v>
+        <v>328.17</v>
       </c>
       <c r="F31" t="n">
-        <v>-348.0621619396069</v>
+        <v>0.6278</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9990213764568128</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0.4566</v>
-      </c>
-      <c r="I31" t="n">
-        <v>0.5664</v>
-      </c>
-      <c r="J31" t="n">
-        <v>111</v>
-      </c>
-      <c r="K31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>328.17</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1605,24 +1471,20 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1039.981562161296</v>
+        <v>314.7</v>
       </c>
       <c r="F32" t="n">
-        <v>-378.4452152884974</v>
+        <v>0.6588000000000001</v>
       </c>
       <c r="G32" t="n">
-        <v>0.9990452546712528</v>
-      </c>
-      <c r="H32" t="n">
-        <v>0.3988</v>
-      </c>
-      <c r="I32" t="n">
-        <v>0.6539</v>
-      </c>
-      <c r="J32" t="n">
-        <v>127</v>
-      </c>
-      <c r="K32" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>314.70, 185.46, 539.01</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1642,24 +1504,20 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>1506.083728710963</v>
+        <v>476.43</v>
       </c>
       <c r="F33" t="n">
-        <v>-1385.653955662049</v>
+        <v>1.23</v>
       </c>
       <c r="G33" t="n">
-        <v>0.9990257910181267</v>
-      </c>
-      <c r="H33" t="n">
-        <v>1.0717</v>
-      </c>
-      <c r="I33" t="n">
-        <v>1.2125</v>
-      </c>
-      <c r="J33" t="n">
-        <v>73</v>
-      </c>
-      <c r="K33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>476.43</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1679,24 +1537,20 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>1114.139390510288</v>
+        <v>212.13</v>
       </c>
       <c r="F34" t="n">
-        <v>-282.8735488409719</v>
+        <v>0.4431</v>
       </c>
       <c r="G34" t="n">
-        <v>0.9990679710150053</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0.3743</v>
-      </c>
-      <c r="I34" t="n">
-        <v>0.4423</v>
-      </c>
-      <c r="J34" t="n">
-        <v>76</v>
-      </c>
-      <c r="K34" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>212.13</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1716,24 +1570,20 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1078.695052921309</v>
+        <v>602.46</v>
       </c>
       <c r="F35" t="n">
-        <v>-286.3300637206808</v>
+        <v>0.8343</v>
       </c>
       <c r="G35" t="n">
-        <v>0.9990001099435334</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.4239</v>
-      </c>
-      <c r="I35" t="n">
-        <v>0.8088</v>
-      </c>
-      <c r="J35" t="n">
-        <v>387</v>
-      </c>
-      <c r="K35" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>602.46</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1753,24 +1603,20 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1049.462784730027</v>
+        <v>225.96</v>
       </c>
       <c r="F36" t="n">
-        <v>-444.3109406259027</v>
+        <v>0.6345</v>
       </c>
       <c r="G36" t="n">
-        <v>0.9990175094612561</v>
-      </c>
-      <c r="H36" t="n">
-        <v>0.5343</v>
-      </c>
-      <c r="I36" t="n">
-        <v>0.6039</v>
-      </c>
-      <c r="J36" t="n">
-        <v>38</v>
-      </c>
-      <c r="K36" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>225.96, 142.50, 182.12, 118.90, 252.82</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1790,24 +1636,20 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>259.1216291862817</v>
+        <v>140.06</v>
       </c>
       <c r="F37" t="n">
-        <v>-98.55987602989488</v>
+        <v>0.7696</v>
       </c>
       <c r="G37" t="n">
-        <v>0.9990448040035439</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.5163</v>
-      </c>
-      <c r="I37" t="n">
-        <v>0.6529</v>
-      </c>
-      <c r="J37" t="n">
-        <v>70</v>
-      </c>
-      <c r="K37" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>140.06, 83.32, 236.50, 384.41</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1827,24 +1669,20 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>658.5383747869937</v>
+        <v>165.11</v>
       </c>
       <c r="F38" t="n">
-        <v>-701.930991614038</v>
+        <v>1.2445</v>
       </c>
       <c r="G38" t="n">
-        <v>0.9991027864788505</v>
-      </c>
-      <c r="H38" t="n">
-        <v>1.1184</v>
-      </c>
-      <c r="I38" t="n">
-        <v>1.1669</v>
-      </c>
-      <c r="J38" t="n">
-        <v>25</v>
-      </c>
-      <c r="K38" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>165.11</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1864,24 +1702,20 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>889.9833720818081</v>
+        <v>712.33</v>
       </c>
       <c r="F39" t="n">
-        <v>-845.9547426133787</v>
+        <v>1.7512</v>
       </c>
       <c r="G39" t="n">
-        <v>0.9990089282994327</v>
-      </c>
-      <c r="H39" t="n">
-        <v>1.2064</v>
-      </c>
-      <c r="I39" t="n">
-        <v>1.7497</v>
-      </c>
-      <c r="J39" t="n">
-        <v>273</v>
-      </c>
-      <c r="K39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>712.33</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1901,24 +1735,20 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>1725.547285022666</v>
+        <v>441.83</v>
       </c>
       <c r="F40" t="n">
-        <v>-1526.757178453126</v>
+        <v>1.1393</v>
       </c>
       <c r="G40" t="n">
-        <v>0.9990088190749582</v>
-      </c>
-      <c r="H40" t="n">
-        <v>1.0063</v>
-      </c>
-      <c r="I40" t="n">
-        <v>1.1361</v>
-      </c>
-      <c r="J40" t="n">
-        <v>69</v>
-      </c>
-      <c r="K40" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>441.83</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1938,24 +1768,20 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>906.2276549502392</v>
+        <v>353.65</v>
       </c>
       <c r="F41" t="n">
-        <v>-649.4963719729707</v>
+        <v>1.1042</v>
       </c>
       <c r="G41" t="n">
-        <v>0.9990255281938976</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0.762</v>
-      </c>
-      <c r="I41" t="n">
-        <v>1.1012</v>
-      </c>
-      <c r="J41" t="n">
-        <v>171</v>
-      </c>
-      <c r="K41" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>353.65</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1975,24 +1801,20 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1215.189428341425</v>
+        <v>590.62</v>
       </c>
       <c r="F42" t="n">
-        <v>-1070.627665727639</v>
+        <v>1.365</v>
       </c>
       <c r="G42" t="n">
-        <v>0.9990481474435704</v>
-      </c>
-      <c r="H42" t="n">
-        <v>1.0506</v>
-      </c>
-      <c r="I42" t="n">
-        <v>1.3636</v>
-      </c>
-      <c r="J42" t="n">
-        <v>156</v>
-      </c>
-      <c r="K42" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>590.62, 19.73</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2012,24 +1834,20 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>1195.049747172969</v>
+        <v>282.37</v>
       </c>
       <c r="F43" t="n">
-        <v>-362.9720232488672</v>
+        <v>0.5377</v>
       </c>
       <c r="G43" t="n">
-        <v>0.9990364389947766</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0.3961</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0.5368000000000001</v>
-      </c>
-      <c r="J43" t="n">
-        <v>142</v>
-      </c>
-      <c r="K43" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>282.37</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2049,24 +1867,20 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>1361.628229446383</v>
+        <v>838.92</v>
       </c>
       <c r="F44" t="n">
-        <v>-925.235372813004</v>
+        <v>1.3325</v>
       </c>
       <c r="G44" t="n">
-        <v>0.9990017788526353</v>
-      </c>
-      <c r="H44" t="n">
-        <v>0.7485000000000001</v>
-      </c>
-      <c r="I44" t="n">
-        <v>1.2519</v>
-      </c>
-      <c r="J44" t="n">
-        <v>254</v>
-      </c>
-      <c r="K44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>838.92</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2086,28 +1900,20 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>617.1036268031388</v>
+        <v>408.45</v>
       </c>
       <c r="F45" t="n">
-        <v>-282.7626415644129</v>
+        <v>1.2064</v>
       </c>
       <c r="G45" t="n">
-        <v>0.9985490975132543</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0.6273</v>
-      </c>
-      <c r="I45" t="n">
-        <v>0.7069</v>
-      </c>
-      <c r="J45" t="n">
-        <v>20</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>NO_WINDOW_MET_R2_THRESHOLD - relaxed to best available, verify manually</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>408.45, 348.32, 410.86, 567.00</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2127,24 +1933,20 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>752.845440412168</v>
+        <v>171.95</v>
       </c>
       <c r="F46" t="n">
-        <v>-306.1342286614628</v>
+        <v>0.6092</v>
       </c>
       <c r="G46" t="n">
-        <v>0.9990380301646603</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0.4533</v>
-      </c>
-      <c r="I46" t="n">
-        <v>0.5478</v>
-      </c>
-      <c r="J46" t="n">
-        <v>99</v>
-      </c>
-      <c r="K46" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>171.95</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2164,24 +1966,20 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>1200.171058508329</v>
+        <v>484.01</v>
       </c>
       <c r="F47" t="n">
-        <v>-720.4033098330844</v>
+        <v>0.973</v>
       </c>
       <c r="G47" t="n">
-        <v>0.9990039121273478</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0.656</v>
-      </c>
-      <c r="I47" t="n">
-        <v>0.8487</v>
-      </c>
-      <c r="J47" t="n">
-        <v>99</v>
-      </c>
-      <c r="K47" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>484.01</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2201,24 +1999,20 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1140.012272637047</v>
+        <v>708.98</v>
       </c>
       <c r="F48" t="n">
-        <v>-714.5089330670205</v>
+        <v>1.2536</v>
       </c>
       <c r="G48" t="n">
-        <v>0.9990443881923791</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0.6353</v>
-      </c>
-      <c r="I48" t="n">
-        <v>1.2519</v>
-      </c>
-      <c r="J48" t="n">
-        <v>309</v>
-      </c>
-      <c r="K48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>708.98</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2238,24 +2032,20 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>1338.194540546541</v>
+        <v>652.41</v>
       </c>
       <c r="F49" t="n">
-        <v>-258.166978188477</v>
+        <v>0.6868</v>
       </c>
       <c r="G49" t="n">
-        <v>0.9990091295384337</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0.2121</v>
-      </c>
-      <c r="I49" t="n">
-        <v>0.6860000000000001</v>
-      </c>
-      <c r="J49" t="n">
-        <v>475</v>
-      </c>
-      <c r="K49" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>652.41</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2275,24 +2065,20 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1848.869026891513</v>
+        <v>932.98</v>
       </c>
       <c r="F50" t="n">
-        <v>-1947.820232789468</v>
+        <v>1.6039</v>
       </c>
       <c r="G50" t="n">
-        <v>0.9990053384080464</v>
-      </c>
-      <c r="H50" t="n">
-        <v>1.1134</v>
-      </c>
-      <c r="I50" t="n">
-        <v>1.483</v>
-      </c>
-      <c r="J50" t="n">
-        <v>191</v>
-      </c>
-      <c r="K50" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>932.98</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2312,24 +2098,20 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1376.153767579717</v>
+        <v>721.97</v>
       </c>
       <c r="F51" t="n">
-        <v>-732.0609683150279</v>
+        <v>1.0569</v>
       </c>
       <c r="G51" t="n">
-        <v>0.999000053475678</v>
-      </c>
-      <c r="H51" t="n">
-        <v>0.6061</v>
-      </c>
-      <c r="I51" t="n">
-        <v>1.0546</v>
-      </c>
-      <c r="J51" t="n">
-        <v>228</v>
-      </c>
-      <c r="K51" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>721.97</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2349,24 +2131,20 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>1915.109840344322</v>
+        <v>455.64</v>
       </c>
       <c r="F52" t="n">
-        <v>-802.2486298840217</v>
+        <v>0.6575</v>
       </c>
       <c r="G52" t="n">
-        <v>0.9990625924918645</v>
-      </c>
-      <c r="H52" t="n">
-        <v>0.5421</v>
-      </c>
-      <c r="I52" t="n">
-        <v>0.6554</v>
-      </c>
-      <c r="J52" t="n">
-        <v>47</v>
-      </c>
-      <c r="K52" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>455.64, 107.63, 106.86, 548.23</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2386,24 +2164,20 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>1545.610382873935</v>
+        <v>661.3200000000001</v>
       </c>
       <c r="F53" t="n">
-        <v>-774.9044005008559</v>
+        <v>0.9261</v>
       </c>
       <c r="G53" t="n">
-        <v>0.9990224183770685</v>
-      </c>
-      <c r="H53" t="n">
-        <v>0.5501</v>
-      </c>
-      <c r="I53" t="n">
-        <v>0.9251</v>
-      </c>
-      <c r="J53" t="n">
-        <v>284</v>
-      </c>
-      <c r="K53" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>661.32</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2423,24 +2197,20 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>2106.572669685413</v>
+        <v>1088.12</v>
       </c>
       <c r="F54" t="n">
-        <v>-588.6341387838703</v>
+        <v>0.8532999999999999</v>
       </c>
       <c r="G54" t="n">
-        <v>0.9990001803591724</v>
-      </c>
-      <c r="H54" t="n">
-        <v>0.3629</v>
-      </c>
-      <c r="I54" t="n">
-        <v>0.6473</v>
-      </c>
-      <c r="J54" t="n">
-        <v>215</v>
-      </c>
-      <c r="K54" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>1088.12</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2460,28 +2230,20 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>168.818547133057</v>
+        <v>133.08</v>
       </c>
       <c r="F55" t="n">
-        <v>-376.7788449956973</v>
+        <v>3.0278</v>
       </c>
       <c r="G55" t="n">
-        <v>0.9945947352990696</v>
-      </c>
-      <c r="H55" t="n">
-        <v>2.3475</v>
-      </c>
-      <c r="I55" t="n">
-        <v>2.4458</v>
-      </c>
-      <c r="J55" t="n">
-        <v>20</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>NO_WINDOW_MET_R2_THRESHOLD - relaxed to best available, verify manually</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>133.08, 299.30, 121.07, 250.32</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2501,24 +2263,20 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>586.6664834997483</v>
+        <v>232.06</v>
       </c>
       <c r="F56" t="n">
-        <v>-106.0124547301793</v>
+        <v>0.5775</v>
       </c>
       <c r="G56" t="n">
-        <v>0.9990162496020367</v>
-      </c>
-      <c r="H56" t="n">
-        <v>0.2452</v>
-      </c>
-      <c r="I56" t="n">
-        <v>0.5765</v>
-      </c>
-      <c r="J56" t="n">
-        <v>248</v>
-      </c>
-      <c r="K56" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>232.06, 218.53, 141.63, 173.16, 280.21</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2538,24 +2296,20 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1167.592933907032</v>
+        <v>306.17</v>
       </c>
       <c r="F57" t="n">
-        <v>-410.4534303241888</v>
+        <v>0.6045</v>
       </c>
       <c r="G57" t="n">
-        <v>0.9990024739157078</v>
-      </c>
-      <c r="H57" t="n">
-        <v>0.4495</v>
-      </c>
-      <c r="I57" t="n">
-        <v>0.5774</v>
-      </c>
-      <c r="J57" t="n">
-        <v>203</v>
-      </c>
-      <c r="K57" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>306.17</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2575,24 +2329,20 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1435.134652675993</v>
+        <v>497.35</v>
       </c>
       <c r="F58" t="n">
-        <v>-1055.253712649487</v>
+        <v>1.0787</v>
       </c>
       <c r="G58" t="n">
-        <v>0.9990011147843477</v>
-      </c>
-      <c r="H58" t="n">
-        <v>0.7812</v>
-      </c>
-      <c r="I58" t="n">
-        <v>1.0768</v>
-      </c>
-      <c r="J58" t="n">
-        <v>223</v>
-      </c>
-      <c r="K58" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>497.35</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2612,24 +2362,20 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>1697.773575030829</v>
+        <v>915.04</v>
       </c>
       <c r="F59" t="n">
-        <v>-899.2097264674709</v>
+        <v>1.1156</v>
       </c>
       <c r="G59" t="n">
-        <v>0.9990008192894919</v>
-      </c>
-      <c r="H59" t="n">
-        <v>0.6402</v>
-      </c>
-      <c r="I59" t="n">
-        <v>0.9584</v>
-      </c>
-      <c r="J59" t="n">
-        <v>238</v>
-      </c>
-      <c r="K59" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>915.04</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2649,24 +2395,20 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>1885.185435308484</v>
+        <v>700.42</v>
       </c>
       <c r="F60" t="n">
-        <v>-1268.219526399547</v>
+        <v>1.0427</v>
       </c>
       <c r="G60" t="n">
-        <v>0.9990265312101554</v>
-      </c>
-      <c r="H60" t="n">
-        <v>0.8708</v>
-      </c>
-      <c r="I60" t="n">
-        <v>1.0413</v>
-      </c>
-      <c r="J60" t="n">
-        <v>134</v>
-      </c>
-      <c r="K60" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>700.42</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2686,24 +2428,20 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1685.317216938266</v>
+        <v>607.4299999999999</v>
       </c>
       <c r="F61" t="n">
-        <v>-1124.672411208784</v>
+        <v>1.0251</v>
       </c>
       <c r="G61" t="n">
-        <v>0.9990053425708654</v>
-      </c>
-      <c r="H61" t="n">
-        <v>0.7622</v>
-      </c>
-      <c r="I61" t="n">
-        <v>1.023</v>
-      </c>
-      <c r="J61" t="n">
-        <v>197</v>
-      </c>
-      <c r="K61" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>607.43, 220.55</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2723,24 +2461,20 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>1970.164900332887</v>
+        <v>705.67</v>
       </c>
       <c r="F62" t="n">
-        <v>-1571.607304853663</v>
+        <v>1.1538</v>
       </c>
       <c r="G62" t="n">
-        <v>0.9990219409320304</v>
-      </c>
-      <c r="H62" t="n">
-        <v>0.9546</v>
-      </c>
-      <c r="I62" t="n">
-        <v>1.1528</v>
-      </c>
-      <c r="J62" t="n">
-        <v>148</v>
-      </c>
-      <c r="K62" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>705.67</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2760,24 +2494,20 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>2239.334146819076</v>
+        <v>972.28</v>
       </c>
       <c r="F63" t="n">
-        <v>-1579.095361624976</v>
+        <v>1.1783</v>
       </c>
       <c r="G63" t="n">
-        <v>0.9990199526058354</v>
-      </c>
-      <c r="H63" t="n">
-        <v>0.7959000000000001</v>
-      </c>
-      <c r="I63" t="n">
-        <v>1.0551</v>
-      </c>
-      <c r="J63" t="n">
-        <v>198</v>
-      </c>
-      <c r="K63" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>972.28</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2797,24 +2527,20 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>2007.23458105333</v>
+        <v>745.78</v>
       </c>
       <c r="F64" t="n">
-        <v>-891.6941413780797</v>
+        <v>0.8158</v>
       </c>
       <c r="G64" t="n">
-        <v>0.9990154921573913</v>
-      </c>
-      <c r="H64" t="n">
-        <v>0.5269</v>
-      </c>
-      <c r="I64" t="n">
-        <v>0.8149</v>
-      </c>
-      <c r="J64" t="n">
-        <v>219</v>
-      </c>
-      <c r="K64" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>745.78</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2834,24 +2560,20 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>1321.305923449721</v>
+        <v>369.68</v>
       </c>
       <c r="F65" t="n">
-        <v>-1042.253151060949</v>
+        <v>1.054</v>
       </c>
       <c r="G65" t="n">
-        <v>0.9990103740003758</v>
-      </c>
-      <c r="H65" t="n">
-        <v>0.8685</v>
-      </c>
-      <c r="I65" t="n">
-        <v>0.9958</v>
-      </c>
-      <c r="J65" t="n">
-        <v>98</v>
-      </c>
-      <c r="K65" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>369.68</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2871,24 +2593,20 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>1635.652842142222</v>
+        <v>588.4</v>
       </c>
       <c r="F66" t="n">
-        <v>-645.9706695949335</v>
+        <v>0.7554</v>
       </c>
       <c r="G66" t="n">
-        <v>0.9990049285631223</v>
-      </c>
-      <c r="H66" t="n">
-        <v>0.459</v>
-      </c>
-      <c r="I66" t="n">
-        <v>0.7544</v>
-      </c>
-      <c r="J66" t="n">
-        <v>225</v>
-      </c>
-      <c r="K66" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>588.40</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2908,24 +2626,20 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>1884.730315024063</v>
+        <v>791.6</v>
       </c>
       <c r="F67" t="n">
-        <v>-346.1636718073766</v>
+        <v>0.6596</v>
       </c>
       <c r="G67" t="n">
-        <v>0.9990042564749072</v>
-      </c>
-      <c r="H67" t="n">
-        <v>0.2847</v>
-      </c>
-      <c r="I67" t="n">
-        <v>0.5562</v>
-      </c>
-      <c r="J67" t="n">
-        <v>203</v>
-      </c>
-      <c r="K67" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>791.60</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2945,24 +2659,20 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>1304.753658025737</v>
+        <v>417.56</v>
       </c>
       <c r="F68" t="n">
-        <v>-458.5073083625758</v>
+        <v>0.6693</v>
       </c>
       <c r="G68" t="n">
-        <v>0.9990341421370107</v>
-      </c>
-      <c r="H68" t="n">
-        <v>0.5075</v>
-      </c>
-      <c r="I68" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="J68" t="n">
-        <v>122</v>
-      </c>
-      <c r="K68" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>417.56, 81.49</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2982,24 +2692,20 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>972.7898680740374</v>
+        <v>266.1</v>
       </c>
       <c r="F69" t="n">
-        <v>-609.8363127494714</v>
+        <v>0.8983</v>
       </c>
       <c r="G69" t="n">
-        <v>0.9990513979307996</v>
-      </c>
-      <c r="H69" t="n">
-        <v>0.7548</v>
-      </c>
-      <c r="I69" t="n">
-        <v>0.897</v>
-      </c>
-      <c r="J69" t="n">
-        <v>104</v>
-      </c>
-      <c r="K69" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>266.10</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3019,24 +2725,20 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>1358.963501943409</v>
+        <v>406.5</v>
       </c>
       <c r="F70" t="n">
-        <v>-1270.091876993143</v>
+        <v>1.2102</v>
       </c>
       <c r="G70" t="n">
-        <v>0.9990033387708966</v>
-      </c>
-      <c r="H70" t="n">
-        <v>0.9966</v>
-      </c>
-      <c r="I70" t="n">
-        <v>1.1378</v>
-      </c>
-      <c r="J70" t="n">
-        <v>111</v>
-      </c>
-      <c r="K70" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>406.50</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3056,24 +2758,20 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>1304.352423354473</v>
+        <v>517.6900000000001</v>
       </c>
       <c r="F71" t="n">
-        <v>-173.7500920599462</v>
+        <v>0.5294</v>
       </c>
       <c r="G71" t="n">
-        <v>0.9990016465160787</v>
-      </c>
-      <c r="H71" t="n">
-        <v>0.1984</v>
-      </c>
-      <c r="I71" t="n">
-        <v>0.5282</v>
-      </c>
-      <c r="J71" t="n">
-        <v>250</v>
-      </c>
-      <c r="K71" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>517.69, 267.12, 237.32, 582.32</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3093,24 +2791,20 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>458.347769076096</v>
+        <v>346.25</v>
       </c>
       <c r="F72" t="n">
-        <v>-144.1136011961289</v>
+        <v>0.8213</v>
       </c>
       <c r="G72" t="n">
-        <v>0.999060862675916</v>
-      </c>
-      <c r="H72" t="n">
-        <v>0.4066</v>
-      </c>
-      <c r="I72" t="n">
-        <v>0.5087</v>
-      </c>
-      <c r="J72" t="n">
-        <v>81</v>
-      </c>
-      <c r="K72" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>346.25</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3130,24 +2824,20 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>1549.445736462649</v>
+        <v>772.05</v>
       </c>
       <c r="F73" t="n">
-        <v>-980.0401700039924</v>
+        <v>1.1346</v>
       </c>
       <c r="G73" t="n">
-        <v>0.9990189689727862</v>
-      </c>
-      <c r="H73" t="n">
-        <v>0.7556</v>
-      </c>
-      <c r="I73" t="n">
-        <v>1.1333</v>
-      </c>
-      <c r="J73" t="n">
-        <v>283</v>
-      </c>
-      <c r="K73" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>772.05</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3167,24 +2857,20 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>1740.168498750401</v>
+        <v>801.27</v>
       </c>
       <c r="F74" t="n">
-        <v>13.65967604729902</v>
+        <v>0.4687</v>
       </c>
       <c r="G74" t="n">
-        <v>0.9990019936169656</v>
-      </c>
-      <c r="H74" t="n">
-        <v>0.0941</v>
-      </c>
-      <c r="I74" t="n">
-        <v>0.4478</v>
-      </c>
-      <c r="J74" t="n">
-        <v>538</v>
-      </c>
-      <c r="K74" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>801.27</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3204,28 +2890,20 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>405.3267636452448</v>
+        <v>37.26</v>
       </c>
       <c r="F75" t="n">
-        <v>-142.8645500334846</v>
+        <v>0.5784</v>
       </c>
       <c r="G75" t="n">
-        <v>0.9835890162016051</v>
-      </c>
-      <c r="H75" t="n">
-        <v>0.3458</v>
-      </c>
-      <c r="I75" t="n">
-        <v>0.3967</v>
-      </c>
-      <c r="J75" t="n">
-        <v>20</v>
-      </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>NO_WINDOW_MET_R2_THRESHOLD - relaxed to best available, verify manually</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>37.26, 697.40</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3245,24 +2923,20 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>1719.959476371546</v>
+        <v>640.4</v>
       </c>
       <c r="F76" t="n">
-        <v>-952.9225720010677</v>
+        <v>0.9232</v>
       </c>
       <c r="G76" t="n">
-        <v>0.9990396170132734</v>
-      </c>
-      <c r="H76" t="n">
-        <v>0.6761</v>
-      </c>
-      <c r="I76" t="n">
-        <v>0.9221</v>
-      </c>
-      <c r="J76" t="n">
-        <v>189</v>
-      </c>
-      <c r="K76" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>640.40</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3282,24 +2956,20 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>1769.866191510748</v>
+        <v>593.67</v>
       </c>
       <c r="F77" t="n">
-        <v>-1031.586993664408</v>
+        <v>0.9154</v>
       </c>
       <c r="G77" t="n">
-        <v>0.9990219076997667</v>
-      </c>
-      <c r="H77" t="n">
-        <v>0.6801</v>
-      </c>
-      <c r="I77" t="n">
-        <v>0.9143</v>
-      </c>
-      <c r="J77" t="n">
-        <v>176</v>
-      </c>
-      <c r="K77" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>593.67</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>